<commit_message>
Update iris exploratory analysis spreadsheet
Replace analise_exploratoria_iris.xlsx with an updated workbook containing revised exploratory analysis for the Iris dataset. The new file includes updated summaries, charts, and formatting improvements to reflect recent analysis changes.
</commit_message>
<xml_diff>
--- a/Bacharelado - Ciência da Computação IMPACTA/5 Semestre/Análise Exploratória de Dados/Atividade Prática 1 - dataset iris/analise_exploratoria_iris.xlsx
+++ b/Bacharelado - Ciência da Computação IMPACTA/5 Semestre/Análise Exploratória de Dados/Atividade Prática 1 - dataset iris/analise_exploratoria_iris.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alunoimpacta-my.sharepoint.com/personal/2401895_alunoimpacta_com_br/Documents/Atividades/5 SEM/Análise Exploratória de Dados/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\git\dev\Bacharelado - Ciência da Computação IMPACTA\5 Semestre\Análise Exploratória de Dados\Atividade Prática 1 - dataset iris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{713CA1CE-0929-4B40-B309-73F39E0AC3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A2D1FD-AF4A-4D36-91C6-7B007C9CCAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B4897A10-BDA1-46D3-9F80-A9497B8F36FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15990" activeTab="1" xr2:uid="{B4897A10-BDA1-46D3-9F80-A9497B8F36FD}"/>
   </bookViews>
   <sheets>
     <sheet name="iris" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="90">
   <si>
     <t>Sepal.Length</t>
   </si>
@@ -302,6 +302,41 @@
   </si>
   <si>
     <t>Frequência Relativa (em porcentagem %):</t>
+  </si>
+  <si>
+    <t>Média</t>
+  </si>
+  <si>
+    <t>Fórmula: AVERAGE = Média.</t>
+  </si>
+  <si>
+    <t>Fórmula: MEDIAN = Mediana.</t>
+  </si>
+  <si>
+    <t>Fórmula: STDEV.S
+ST → Standard
+DEV → Deviation
+S → Sample
+Standard Deviation (Sample)
+Desvio padrão amostral</t>
+  </si>
+  <si>
+    <t>Fórmula: VAR.S
+VAR → Variance
+S → Sample
+Variância amostral</t>
+  </si>
+  <si>
+    <t>Média Total</t>
+  </si>
+  <si>
+    <t>Mediana Total</t>
+  </si>
+  <si>
+    <t>Desvio padrão Total</t>
+  </si>
+  <si>
+    <t>Variância Total</t>
   </si>
 </sst>
 </file>
@@ -340,8 +375,9 @@
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -394,7 +430,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -418,57 +454,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
@@ -477,8 +463,23 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
@@ -486,82 +487,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -570,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -578,71 +511,59 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -659,6 +580,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>134086</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>881808</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>123903</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4A1EEB1-056D-6E6B-CBF4-2CD048935BDC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6786932" y="5335465"/>
+          <a:ext cx="1549861" cy="562053"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>140426</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>71805</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>875468</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>30746</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B76E795-FB87-C33E-79CF-C791A47D122B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6793272" y="6035920"/>
+          <a:ext cx="1537181" cy="530441"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -979,16 +993,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88618352-996F-4924-958C-5F95E10577E8}">
   <dimension ref="A1:E151"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1005,7 +1018,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1022,7 +1035,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1039,7 +1052,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1056,7 +1069,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1073,7 +1086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1090,7 +1103,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1107,7 +1120,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -1124,7 +1137,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -1141,7 +1154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -1158,7 +1171,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -1175,7 +1188,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
@@ -1192,7 +1205,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
@@ -1209,7 +1222,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>28</v>
       </c>
@@ -1226,7 +1239,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>30</v>
       </c>
@@ -1243,7 +1256,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
@@ -1260,7 +1273,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -1277,7 +1290,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
@@ -1294,7 +1307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>5</v>
       </c>
@@ -1311,7 +1324,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>34</v>
       </c>
@@ -1328,7 +1341,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>5</v>
       </c>
@@ -1345,7 +1358,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -1362,7 +1375,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>5</v>
       </c>
@@ -1379,7 +1392,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
@@ -1396,7 +1409,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>5</v>
       </c>
@@ -1413,7 +1426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>28</v>
       </c>
@@ -1430,7 +1443,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>5</v>
       </c>
@@ -1447,7 +1460,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>5</v>
       </c>
@@ -1464,7 +1477,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>39</v>
       </c>
@@ -1481,7 +1494,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -1498,7 +1511,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>11</v>
       </c>
@@ -1515,7 +1528,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
@@ -1532,7 +1545,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>18</v>
       </c>
@@ -1549,7 +1562,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>39</v>
       </c>
@@ -1566,7 +1579,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>41</v>
       </c>
@@ -1583,7 +1596,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>10</v>
       </c>
@@ -1600,7 +1613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>5</v>
       </c>
@@ -1617,7 +1630,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>41</v>
       </c>
@@ -1634,7 +1647,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>10</v>
       </c>
@@ -1651,7 +1664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>24</v>
       </c>
@@ -1668,7 +1681,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>5</v>
       </c>
@@ -1685,7 +1698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>5</v>
       </c>
@@ -1702,7 +1715,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
@@ -1719,7 +1732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>24</v>
       </c>
@@ -1736,7 +1749,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>5</v>
       </c>
@@ -1753,7 +1766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>5</v>
       </c>
@@ -1770,7 +1783,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>28</v>
       </c>
@@ -1787,7 +1800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>5</v>
       </c>
@@ -1804,7 +1817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>14</v>
       </c>
@@ -1821,7 +1834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>46</v>
       </c>
@@ -1838,7 +1851,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>5</v>
       </c>
@@ -1855,7 +1868,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>7</v>
       </c>
@@ -1872,7 +1885,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>48</v>
       </c>
@@ -1889,7 +1902,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>49</v>
       </c>
@@ -1906,7 +1919,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>41</v>
       </c>
@@ -1923,7 +1936,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>50</v>
       </c>
@@ -1940,7 +1953,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>34</v>
       </c>
@@ -1957,7 +1970,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>52</v>
       </c>
@@ -1974,7 +1987,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>10</v>
       </c>
@@ -1991,7 +2004,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>54</v>
       </c>
@@ -2008,7 +2021,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>39</v>
       </c>
@@ -2025,7 +2038,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>5</v>
       </c>
@@ -2042,7 +2055,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>56</v>
       </c>
@@ -2059,7 +2072,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>6</v>
       </c>
@@ -2076,7 +2089,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>58</v>
       </c>
@@ -2093,7 +2106,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>59</v>
       </c>
@@ -2110,7 +2123,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>60</v>
       </c>
@@ -2127,7 +2140,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>59</v>
       </c>
@@ -2144,7 +2157,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>32</v>
       </c>
@@ -2161,7 +2174,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>61</v>
       </c>
@@ -2178,7 +2191,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>59</v>
       </c>
@@ -2195,7 +2208,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>56</v>
       </c>
@@ -2212,7 +2225,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>58</v>
       </c>
@@ -2229,7 +2242,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>52</v>
       </c>
@@ -2246,7 +2259,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>58</v>
       </c>
@@ -2263,7 +2276,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>48</v>
       </c>
@@ -2280,7 +2293,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>54</v>
       </c>
@@ -2297,7 +2310,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>64</v>
       </c>
@@ -2314,7 +2327,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>60</v>
       </c>
@@ -2331,7 +2344,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>6</v>
       </c>
@@ -2348,7 +2361,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>34</v>
       </c>
@@ -2365,7 +2378,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="82" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>41</v>
       </c>
@@ -2382,7 +2395,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>41</v>
       </c>
@@ -2399,7 +2412,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>32</v>
       </c>
@@ -2416,7 +2429,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>6</v>
       </c>
@@ -2433,7 +2446,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>18</v>
       </c>
@@ -2450,7 +2463,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>6</v>
       </c>
@@ -2467,7 +2480,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>60</v>
       </c>
@@ -2484,7 +2497,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>52</v>
       </c>
@@ -2501,7 +2514,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>59</v>
       </c>
@@ -2518,7 +2531,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>41</v>
       </c>
@@ -2535,7 +2548,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>41</v>
       </c>
@@ -2552,7 +2565,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>58</v>
       </c>
@@ -2569,7 +2582,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>32</v>
       </c>
@@ -2586,7 +2599,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>5</v>
       </c>
@@ -2603,7 +2616,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>59</v>
       </c>
@@ -2620,7 +2633,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>34</v>
       </c>
@@ -2637,7 +2650,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>34</v>
       </c>
@@ -2654,7 +2667,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>61</v>
       </c>
@@ -2671,7 +2684,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>5</v>
       </c>
@@ -2688,7 +2701,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>34</v>
       </c>
@@ -2705,7 +2718,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>52</v>
       </c>
@@ -2722,7 +2735,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>32</v>
       </c>
@@ -2739,7 +2752,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>67</v>
       </c>
@@ -2756,7 +2769,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>52</v>
       </c>
@@ -2773,7 +2786,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>50</v>
       </c>
@@ -2790,7 +2803,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>69</v>
       </c>
@@ -2807,7 +2820,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>10</v>
       </c>
@@ -2824,7 +2837,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>70</v>
       </c>
@@ -2841,7 +2854,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>60</v>
       </c>
@@ -2858,7 +2871,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>71</v>
       </c>
@@ -2875,7 +2888,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>50</v>
       </c>
@@ -2892,7 +2905,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>48</v>
       </c>
@@ -2909,7 +2922,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>64</v>
       </c>
@@ -2926,7 +2939,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>34</v>
       </c>
@@ -2943,7 +2956,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>32</v>
       </c>
@@ -2960,7 +2973,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>48</v>
       </c>
@@ -2977,7 +2990,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>50</v>
       </c>
@@ -2994,7 +3007,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>72</v>
       </c>
@@ -3011,7 +3024,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>72</v>
       </c>
@@ -3028,7 +3041,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>6</v>
       </c>
@@ -3045,7 +3058,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>49</v>
       </c>
@@ -3062,7 +3075,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>59</v>
       </c>
@@ -3079,7 +3092,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>72</v>
       </c>
@@ -3096,7 +3109,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>52</v>
       </c>
@@ -3113,7 +3126,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="126" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>60</v>
       </c>
@@ -3130,7 +3143,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="127" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>71</v>
       </c>
@@ -3147,7 +3160,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="128" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>61</v>
       </c>
@@ -3164,7 +3177,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="129" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>58</v>
       </c>
@@ -3181,7 +3194,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="130" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>48</v>
       </c>
@@ -3198,7 +3211,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="131" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>71</v>
       </c>
@@ -3215,7 +3228,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="132" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>73</v>
       </c>
@@ -3232,7 +3245,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="133" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>74</v>
       </c>
@@ -3249,7 +3262,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="134" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>48</v>
       </c>
@@ -3266,7 +3279,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="135" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>52</v>
       </c>
@@ -3283,7 +3296,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="136" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>58</v>
       </c>
@@ -3300,7 +3313,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="137" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>72</v>
       </c>
@@ -3317,7 +3330,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="138" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>52</v>
       </c>
@@ -3334,7 +3347,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="139" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>48</v>
       </c>
@@ -3351,7 +3364,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="140" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>6</v>
       </c>
@@ -3368,7 +3381,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="141" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>49</v>
       </c>
@@ -3385,7 +3398,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="142" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>60</v>
       </c>
@@ -3402,7 +3415,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="143" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>49</v>
       </c>
@@ -3419,7 +3432,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="144" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>32</v>
       </c>
@@ -3436,7 +3449,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="145" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>64</v>
       </c>
@@ -3453,7 +3466,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="146" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>60</v>
       </c>
@@ -3470,7 +3483,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="147" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>60</v>
       </c>
@@ -3487,7 +3500,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="148" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>52</v>
       </c>
@@ -3504,7 +3517,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="149" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>50</v>
       </c>
@@ -3521,7 +3534,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="150" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>61</v>
       </c>
@@ -3538,7 +3551,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="151" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>56</v>
       </c>
@@ -3562,159 +3575,459 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9669B12D-02B7-4126-86EB-6ECFB1A6D83E}">
-  <dimension ref="B1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:G38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="20.77734375" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="10" t="s">
+    <row r="2" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="12"/>
-    </row>
-    <row r="3" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="14" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="3" t="str" cm="1">
+      <c r="C3" s="4"/>
+      <c r="D3" s="5" t="str" cm="1">
         <f t="array" ref="D3:D5">_xlfn.UNIQUE(iris!E2:E151)</f>
         <v>setosa</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="13"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="4" t="str">
+      <c r="F3" t="str" cm="1">
+        <f t="array" ref="F3:F7">(TRANSPOSE(iris!A1:E1))</f>
+        <v>Sepal.Length</v>
+      </c>
+      <c r="G3" t="str">
+        <f>(_xlfn.TRANSLATE(F3))</f>
+        <v>Sepal.Comprimento</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="6" t="str">
         <v>versicolor</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="5" t="str">
+      <c r="F4" t="str">
+        <v>Sepal.Width</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" ref="G4:G7" si="0">(_xlfn.TRANSLATE(F4))</f>
+        <v>Sepal.Width</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="7" t="str">
         <v>virginica</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="20" t="s">
+      <c r="F5" t="str">
+        <v>Petal.Length</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="0"/>
+        <v>Pétala. Comprimento</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="C6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="5">
         <f>COUNTIF(iris!E2:E151,'Análise do Dataset Iris'!C6)</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="19"/>
-      <c r="C7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="24">
+      <c r="F6" t="str">
+        <v>Petal.Width</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="0"/>
+        <v>Pétala. Largura</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="12">
         <f>COUNTIF(iris!E2:E151,'Análise do Dataset Iris'!C7)</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="21"/>
-      <c r="C8" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="5">
+      <c r="F7" t="str">
+        <v>Species</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="0"/>
+        <v>Espécies</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="4"/>
+      <c r="C8" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="7">
         <f>COUNTIF(iris!E2:E153,'Análise do Dataset Iris'!C8)</f>
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="22" t="s">
+    <row r="9" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="6">
+      <c r="C9" s="4"/>
+      <c r="D9" s="8">
         <f>(COUNTA(iris!E1:E150))</f>
         <v>150</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="20" t="s">
+    <row r="10" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="3">
+      <c r="C10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="5">
         <f>D6/$D$9</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="19"/>
-      <c r="C11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="4">
+    <row r="11" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="4"/>
+      <c r="C11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="6">
         <f>D7/$D$9</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="21"/>
-      <c r="C12" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" s="5">
+    <row r="12" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="4"/>
+      <c r="C12" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="7">
         <f>D8/$D$9</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="20" t="s">
+    <row r="13" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="7">
+      <c r="C13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="9">
         <f>D10</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="19"/>
-      <c r="C14" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="8">
+    <row r="14" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+      <c r="C14" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="10">
         <f>D11</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="21"/>
-      <c r="C15" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="9">
+    <row r="15" spans="2:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="4"/>
+      <c r="C15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="11">
         <f>D12</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="8" t="str" cm="1">
+        <f t="array" ref="C16:C19">TRANSPOSE(iris!$A$1:'iris'!$D$1)</f>
+        <v>Sepal.Length</v>
+      </c>
+      <c r="D16" s="8">
+        <f>(AVERAGE(iris!A2:A151))</f>
+        <v>5.4705882352941178</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+      <c r="C17" s="8" t="str">
+        <v>Sepal.Width</v>
+      </c>
+      <c r="D17" s="8">
+        <f>(AVERAGE(iris!B2:B151))</f>
+        <v>3</v>
+      </c>
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="4"/>
+      <c r="C18" s="8" t="str">
+        <v>Petal.Length</v>
+      </c>
+      <c r="D18" s="8">
+        <f>(AVERAGE(iris!C2:C151))</f>
+        <v>4.3076923076923075</v>
+      </c>
+      <c r="E18" s="15"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="4"/>
+      <c r="C19" s="8" t="str">
+        <v>Petal.Width</v>
+      </c>
+      <c r="D19" s="8">
+        <f>(AVERAGE(iris!D2:D151))</f>
+        <v>1.4615384615384615</v>
+      </c>
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8">
+        <f>AVERAGEIF(iris!E2:E151,"setosa",iris!C2:C151)</f>
+        <v>1</v>
+      </c>
+      <c r="E20" s="17"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="19"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8">
+        <f>AVERAGEIF(iris!E2:E151,"versicolor",iris!C2:C151)</f>
+        <v>4</v>
+      </c>
+      <c r="E21" s="17"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="20"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8">
+        <f>AVERAGEIF(iris!E2:E151,"virginica",iris!C2:C151)</f>
+        <v>5.4</v>
+      </c>
+      <c r="E22" s="17"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="8" t="str" cm="1">
+        <f t="array" ref="C23:C26">TRANSPOSE(iris!$A$1:'iris'!$D$1)</f>
+        <v>Sepal.Length</v>
+      </c>
+      <c r="D23" s="8">
+        <f>(MEDIAN(iris!A2:A151))</f>
+        <v>5</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="4"/>
+      <c r="C24" s="8" t="str">
+        <v>Sepal.Width</v>
+      </c>
+      <c r="D24" s="8">
+        <f>(MEDIAN(iris!B2:B151))</f>
+        <v>3</v>
+      </c>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="4"/>
+      <c r="C25" s="8" t="str">
+        <v>Petal.Length</v>
+      </c>
+      <c r="D25" s="8">
+        <f>(MEDIAN(iris!C2:C151))</f>
+        <v>4</v>
+      </c>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="4"/>
+      <c r="C26" s="8" t="str">
+        <v>Petal.Width</v>
+      </c>
+      <c r="D26" s="8">
+        <f>(MEDIAN(iris!D2:D151))</f>
+        <v>1</v>
+      </c>
+      <c r="E26" s="15"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="13"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="17"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="13"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="17"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="13"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="17"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="13"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="17"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="8" t="str" cm="1">
+        <f t="array" ref="C31:C34">TRANSPOSE(iris!$A$1:'iris'!$D$1)</f>
+        <v>Sepal.Length</v>
+      </c>
+      <c r="D31" s="8">
+        <f>(_xlfn.STDEV.S(iris!A2:A151))</f>
+        <v>0.62426427284679842</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="4"/>
+      <c r="C32" s="8" t="str">
+        <v>Sepal.Width</v>
+      </c>
+      <c r="D32" s="8">
+        <f>(_xlfn.STDEV.S(iris!B2:B151))</f>
+        <v>0.27216552697590868</v>
+      </c>
+      <c r="E32" s="14"/>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="4"/>
+      <c r="C33" s="8" t="str">
+        <v>Petal.Length</v>
+      </c>
+      <c r="D33" s="8">
+        <f>(_xlfn.STDEV.S(iris!C2:C151))</f>
+        <v>1.315587028960544</v>
+      </c>
+      <c r="E33" s="14"/>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="4"/>
+      <c r="C34" s="8" t="str">
+        <v>Petal.Width</v>
+      </c>
+      <c r="D34" s="8">
+        <f>(_xlfn.STDEV.S(iris!D2:D151))</f>
+        <v>0.5188745216627707</v>
+      </c>
+      <c r="E34" s="14"/>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C35" s="8" t="str" cm="1">
+        <f t="array" ref="C35:C38">TRANSPOSE(iris!$A$1:'iris'!$D$1)</f>
+        <v>Sepal.Length</v>
+      </c>
+      <c r="D35" s="8">
+        <f>(_xlfn.VAR.S(iris!A2:A151))</f>
+        <v>0.38970588235294201</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36" s="4"/>
+      <c r="C36" s="8" t="str">
+        <v>Sepal.Width</v>
+      </c>
+      <c r="D36" s="8">
+        <f>(_xlfn.VAR.S(iris!B2:B151))</f>
+        <v>7.407407407407407E-2</v>
+      </c>
+      <c r="E36" s="14"/>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B37" s="4"/>
+      <c r="C37" s="8" t="str">
+        <v>Petal.Length</v>
+      </c>
+      <c r="D37" s="8">
+        <f>(_xlfn.VAR.S(iris!C2:C151))</f>
+        <v>1.7307692307692311</v>
+      </c>
+      <c r="E37" s="14"/>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B38" s="4"/>
+      <c r="C38" s="8" t="str">
+        <v>Petal.Width</v>
+      </c>
+      <c r="D38" s="8">
+        <f>(_xlfn.VAR.S(iris!D2:D151))</f>
+        <v>0.26923076923076916</v>
+      </c>
+      <c r="E38" s="14"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="15">
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E23:E26"/>
+    <mergeCell ref="E31:E34"/>
+    <mergeCell ref="E35:E38"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="B31:B34"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:C5"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B13:B15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>